<commit_message>
Clean up Excel header styling without blue background fills
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -14804,7 +14804,7 @@
         <v>48</v>
       </c>
       <c r="E18" t="n">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="F18" t="n">
         <v>42</v>
@@ -14848,7 +14848,7 @@
         <v>56</v>
       </c>
       <c r="E20" t="n">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="F20" t="n">
         <v>49</v>
@@ -14870,7 +14870,7 @@
         <v>168</v>
       </c>
       <c r="E21" t="n">
-        <v>372</v>
+        <v>274</v>
       </c>
       <c r="F21" t="n">
         <v>145</v>

</xml_diff>

<commit_message>
feat(hardware): execute live VQE evaluation on IBM Quantum ibm_fez (Job ID daor3p5r85ps73ffmvn0)
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -17100,7 +17100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -17134,7 +17134,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Noisy Simulation (fake_fez Aer Noise Model)</t>
+          <t>Evaluated on Physical IBM Quantum QPU (ibm_fez)</t>
         </is>
       </c>
     </row>
@@ -17146,7 +17146,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>fake_fez</t>
+          <t>ibm_fez</t>
         </is>
       </c>
     </row>
@@ -17158,7 +17158,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sim-aer-noise-001</t>
+          <t>daor3p5r85ps73ffmvn0</t>
         </is>
       </c>
     </row>
@@ -17187,175 +17187,165 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Transpiled 2-Qubit Gate Count (unbound)</t>
+          <t>Transpiled 2-Qubit Gate Count</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Transpiled 2-Qubit Gate Count (bound theta=0)</t>
+          <t>Circuit Depth</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Circuit Depth</t>
+          <t>Exact Active Ground Energy (Ha)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>-639.724283227178</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Exact Active Ground Energy (Ha)</t>
+          <t>Measured Energy (Ha)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-639.724283227178</v>
+        <v>-639.7236460864065</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Measured Energy (Ha)</t>
+          <t>Energy Error (mHa)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-639.7241993565215</v>
+        <v>0.6371407715732857</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Energy Error (mHa)</t>
+          <t>Shots</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.08387065656734194</v>
+        <v>4096</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shots</t>
+          <t>QPU Runtime (seconds)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4096</v>
+        <v>30.35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Simulation Time (s)</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1.767</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Historical Job d330j9cve01c738t02j0</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>UNVERIFIED - confirm in IBM Quantum dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
+          <t>Direct Job Dashboard</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://quantum.ibm.com/jobs/daor3p5r85ps73ffmvn0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Parameter Binding Transpilation Analysis at θ = 0</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+    </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Parameter Binding Transpilation Analysis at θ = 0</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Value</t>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>fake_fez</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>backend</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>fake_fez</t>
-        </is>
+          <t>unbound_depth</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>157</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>unbound_depth</t>
+          <t>unbound_2q_gates</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>157</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>unbound_2q_gates</t>
+          <t>bound_zero_depth</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>bound_zero_depth</t>
+          <t>bound_zero_2q_gates</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>bound_zero_2q_gates</t>
+          <t>gate_reduction_at_zero</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>gate_reduction_at_zero</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix benchmark caching, Excel hardware export, and QPU submission scripts
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,16 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Results" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Results (2e, 2o)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Results (4e, 4o)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Results (6e, 6o)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Active Space Scaling" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Convergence" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Summary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Robustness" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Hardware" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Verification" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Results (2e, 2o)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Results (4e, 4o)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Results (6e, 6o)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Active Space Scaling" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Convergence" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Robustness" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Hardware" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Verification" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2121,397 +2120,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>IBM Quantum Device Calibrated Noisy Simulation &amp; Hardware Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Metric / Parameter</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Evaluated on Physical IBM Quantum QPU (ibm_fez)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Evaluated on Physical IBM Quantum QPU (ibm_fez)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Target Backend</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ibm_fez</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Target Backend</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ibm_fez</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Job ID</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>daqkle3t55cs738rsfrg</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Job ID</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>daqkle3t55cs738rsfrg</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Ansatz Selected</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DexcG (theta sweep [-0.10, +0.10])</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Ansatz Selected</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DexcG (theta sweep [-0.10, +0.10])</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Parameters Optimized</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Parameters Optimized</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Transpiled 2-Qubit Gate Count</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Transpiled 2-Qubit Gate Count</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Circuit Depth</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Circuit Depth</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Exact Active Ground Energy (Ha)</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>-639.7242832271774</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Exact Active Ground Energy (Ha)</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>-639.7242832271774</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Measured Energy (Ha)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Measured Energy (Ha)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Energy Error (mHa)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Energy Error (mHa)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Shots</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>4096</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Shots</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>4096</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>QPU Runtime (seconds)</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>QPU Runtime (seconds)</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Direct Job Dashboard</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>https://quantum.ibm.com/jobs/daqkle3t55cs738rsfrg</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Direct Job Dashboard</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>https://quantum.ibm.com/jobs/daqkle3t55cs738rsfrg</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Parameter Binding Transpilation Analysis at θ = 0</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>backend</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>fake_fez</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>unbound_depth</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>unbound_2q_gates</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>bound_zero_depth</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>bound_zero_2q_gates</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>gate_reduction_at_zero</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3211,20 +2819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N130"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6515,3291 +6110,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Config ID</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Ansatz</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Initialization</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Optimizer</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Parameters</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Final Energy (Ha)</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>Best Energy (Ha)</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>Exact Energy (Ha)</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Error (mHa)</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>Rel Error (%)</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>% Correlation Recovered</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>Total Evaluations</t>
-        </is>
-      </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>Wall Time (s)</t>
-        </is>
-      </c>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>Iterations</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>1</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E67" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" t="n">
-        <v>-639.7242830138499</v>
-      </c>
-      <c r="G67" t="n">
-        <v>-639.7242830138501</v>
-      </c>
-      <c r="H67" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I67" t="n">
-        <v>0.0002133281213900773</v>
-      </c>
-      <c r="J67" t="n">
-        <v>3.334688505396636e-08</v>
-      </c>
-      <c r="K67" t="n">
-        <v>0.9947880592540834</v>
-      </c>
-      <c r="L67" t="n">
-        <v>151</v>
-      </c>
-      <c r="M67" t="n">
-        <v>1.269454400000086</v>
-      </c>
-      <c r="N67" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>2</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E68" t="n">
-        <v>1</v>
-      </c>
-      <c r="F68" t="n">
-        <v>-639.7242749233669</v>
-      </c>
-      <c r="G68" t="n">
-        <v>-639.724282984667</v>
-      </c>
-      <c r="H68" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I68" t="n">
-        <v>0.00830381111427414</v>
-      </c>
-      <c r="J68" t="n">
-        <v>1.298029687474799e-06</v>
-      </c>
-      <c r="K68" t="n">
-        <v>0.7971248646879381</v>
-      </c>
-      <c r="L68" t="n">
-        <v>151</v>
-      </c>
-      <c r="M68" t="n">
-        <v>1.271910199999638</v>
-      </c>
-      <c r="N68" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="n">
-        <v>3</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E69" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" t="n">
-        <v>-639.7242830138499</v>
-      </c>
-      <c r="G69" t="n">
-        <v>-639.7242830138501</v>
-      </c>
-      <c r="H69" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I69" t="n">
-        <v>0.0002133281213900773</v>
-      </c>
-      <c r="J69" t="n">
-        <v>3.334688505396636e-08</v>
-      </c>
-      <c r="K69" t="n">
-        <v>0.9947880592540834</v>
-      </c>
-      <c r="L69" t="n">
-        <v>153</v>
-      </c>
-      <c r="M69" t="n">
-        <v>1.26044789999969</v>
-      </c>
-      <c r="N69" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="n">
-        <v>4</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E70" t="n">
-        <v>1</v>
-      </c>
-      <c r="F70" t="n">
-        <v>-639.7242830138503</v>
-      </c>
-      <c r="G70" t="n">
-        <v>-639.7242830138503</v>
-      </c>
-      <c r="H70" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I70" t="n">
-        <v>0.0002133277803295641</v>
-      </c>
-      <c r="J70" t="n">
-        <v>3.334683174029326e-08</v>
-      </c>
-      <c r="K70" t="n">
-        <v>0.994788067586727</v>
-      </c>
-      <c r="L70" t="n">
-        <v>179</v>
-      </c>
-      <c r="M70" t="n">
-        <v>4.973930999999993</v>
-      </c>
-      <c r="N70" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="n">
-        <v>5</v>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E71" t="n">
-        <v>1</v>
-      </c>
-      <c r="F71" t="n">
-        <v>-639.7242830138501</v>
-      </c>
-      <c r="G71" t="n">
-        <v>-639.7242830138501</v>
-      </c>
-      <c r="H71" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I71" t="n">
-        <v>0.0002133278940164018</v>
-      </c>
-      <c r="J71" t="n">
-        <v>3.334684951151762e-08</v>
-      </c>
-      <c r="K71" t="n">
-        <v>0.9947880648091791</v>
-      </c>
-      <c r="L71" t="n">
-        <v>151</v>
-      </c>
-      <c r="M71" t="n">
-        <v>1.33647000000019</v>
-      </c>
-      <c r="N71" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="n">
-        <v>6</v>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E72" t="n">
-        <v>1</v>
-      </c>
-      <c r="F72" t="n">
-        <v>-639.7241707717523</v>
-      </c>
-      <c r="G72" t="n">
-        <v>-639.7242828206932</v>
-      </c>
-      <c r="H72" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I72" t="n">
-        <v>0.1124554257785348</v>
-      </c>
-      <c r="J72" t="n">
-        <v>1.757873332730748e-05</v>
-      </c>
-      <c r="K72" t="n">
-        <v>-1.747462509374536</v>
-      </c>
-      <c r="L72" t="n">
-        <v>151</v>
-      </c>
-      <c r="M72" t="n">
-        <v>1.426167999999961</v>
-      </c>
-      <c r="N72" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="n">
-        <v>7</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E73" t="n">
-        <v>1</v>
-      </c>
-      <c r="F73" t="n">
-        <v>-639.7242830137131</v>
-      </c>
-      <c r="G73" t="n">
-        <v>-639.7242830137131</v>
-      </c>
-      <c r="H73" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I73" t="n">
-        <v>0.0002134648866558564</v>
-      </c>
-      <c r="J73" t="n">
-        <v>3.336826383688346e-08</v>
-      </c>
-      <c r="K73" t="n">
-        <v>0.9947847178640375</v>
-      </c>
-      <c r="L73" t="n">
-        <v>153</v>
-      </c>
-      <c r="M73" t="n">
-        <v>1.604539100000238</v>
-      </c>
-      <c r="N73" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="n">
-        <v>8</v>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E74" t="n">
-        <v>1</v>
-      </c>
-      <c r="F74" t="n">
-        <v>-639.7242830136666</v>
-      </c>
-      <c r="G74" t="n">
-        <v>-639.7242830136666</v>
-      </c>
-      <c r="H74" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I74" t="n">
-        <v>0.0002135113845724845</v>
-      </c>
-      <c r="J74" t="n">
-        <v>3.337553226765079e-08</v>
-      </c>
-      <c r="K74" t="n">
-        <v>0.9947835818469728</v>
-      </c>
-      <c r="L74" t="n">
-        <v>179</v>
-      </c>
-      <c r="M74" t="n">
-        <v>5.084056600000167</v>
-      </c>
-      <c r="N74" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="n">
-        <v>9</v>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E75" t="n">
-        <v>1</v>
-      </c>
-      <c r="F75" t="n">
-        <v>-639.7242830138497</v>
-      </c>
-      <c r="G75" t="n">
-        <v>-639.7242830138499</v>
-      </c>
-      <c r="H75" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I75" t="n">
-        <v>0.0002133283487637527</v>
-      </c>
-      <c r="J75" t="n">
-        <v>3.33469205964151e-08</v>
-      </c>
-      <c r="K75" t="n">
-        <v>0.9947880536989878</v>
-      </c>
-      <c r="L75" t="n">
-        <v>151</v>
-      </c>
-      <c r="M75" t="n">
-        <v>1.322802700000011</v>
-      </c>
-      <c r="N75" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>10</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E76" t="n">
-        <v>1</v>
-      </c>
-      <c r="F76" t="n">
-        <v>-639.723673395505</v>
-      </c>
-      <c r="G76" t="n">
-        <v>-639.7242816301389</v>
-      </c>
-      <c r="H76" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I76" t="n">
-        <v>0.6098316730458464</v>
-      </c>
-      <c r="J76" t="n">
-        <v>9.532726661077578e-05</v>
-      </c>
-      <c r="K76" t="n">
-        <v>-13.89914467997528</v>
-      </c>
-      <c r="L76" t="n">
-        <v>151</v>
-      </c>
-      <c r="M76" t="n">
-        <v>1.33096149999983</v>
-      </c>
-      <c r="N76" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="n">
-        <v>11</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>1</v>
-      </c>
-      <c r="F77" t="n">
-        <v>-639.7242830124582</v>
-      </c>
-      <c r="G77" t="n">
-        <v>-639.7242830124582</v>
-      </c>
-      <c r="H77" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I77" t="n">
-        <v>0.0002147198756574653</v>
-      </c>
-      <c r="J77" t="n">
-        <v>3.356444038270379e-08</v>
-      </c>
-      <c r="K77" t="n">
-        <v>0.9947540565134826</v>
-      </c>
-      <c r="L77" t="n">
-        <v>153</v>
-      </c>
-      <c r="M77" t="n">
-        <v>1.627792899999804</v>
-      </c>
-      <c r="N77" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>12</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E78" t="n">
-        <v>1</v>
-      </c>
-      <c r="F78" t="n">
-        <v>-639.724283012599</v>
-      </c>
-      <c r="G78" t="n">
-        <v>-639.724283012599</v>
-      </c>
-      <c r="H78" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I78" t="n">
-        <v>0.0002145790176655282</v>
-      </c>
-      <c r="J78" t="n">
-        <v>3.354242183570937e-08</v>
-      </c>
-      <c r="K78" t="n">
-        <v>0.9947574978952506</v>
-      </c>
-      <c r="L78" t="n">
-        <v>179</v>
-      </c>
-      <c r="M78" t="n">
-        <v>5.690470600000026</v>
-      </c>
-      <c r="N78" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>13</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>1</v>
-      </c>
-      <c r="F79" t="n">
-        <v>-639.7242830138498</v>
-      </c>
-      <c r="G79" t="n">
-        <v>-639.7242830138498</v>
-      </c>
-      <c r="H79" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I79" t="n">
-        <v>0.000213328235076915</v>
-      </c>
-      <c r="J79" t="n">
-        <v>3.334690282519074e-08</v>
-      </c>
-      <c r="K79" t="n">
-        <v>0.9947880564765357</v>
-      </c>
-      <c r="L79" t="n">
-        <v>151</v>
-      </c>
-      <c r="M79" t="n">
-        <v>1.316229699999894</v>
-      </c>
-      <c r="N79" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>14</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E80" t="n">
-        <v>1</v>
-      </c>
-      <c r="F80" t="n">
-        <v>-639.7239229370974</v>
-      </c>
-      <c r="G80" t="n">
-        <v>-639.7242776959463</v>
-      </c>
-      <c r="H80" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I80" t="n">
-        <v>0.3602900806072284</v>
-      </c>
-      <c r="J80" t="n">
-        <v>5.631958799339226e-05</v>
-      </c>
-      <c r="K80" t="n">
-        <v>-7.802452012562971</v>
-      </c>
-      <c r="L80" t="n">
-        <v>151</v>
-      </c>
-      <c r="M80" t="n">
-        <v>1.010585900000024</v>
-      </c>
-      <c r="N80" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>15</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E81" t="n">
-        <v>1</v>
-      </c>
-      <c r="F81" t="n">
-        <v>-639.7242830137806</v>
-      </c>
-      <c r="G81" t="n">
-        <v>-639.7242830137806</v>
-      </c>
-      <c r="H81" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I81" t="n">
-        <v>0.0002133974703610875</v>
-      </c>
-      <c r="J81" t="n">
-        <v>3.335772550083206e-08</v>
-      </c>
-      <c r="K81" t="n">
-        <v>0.9947863649499039</v>
-      </c>
-      <c r="L81" t="n">
-        <v>153</v>
-      </c>
-      <c r="M81" t="n">
-        <v>1.500574000000142</v>
-      </c>
-      <c r="N81" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>16</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>DexcG</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E82" t="n">
-        <v>1</v>
-      </c>
-      <c r="F82" t="n">
-        <v>-639.7242830137967</v>
-      </c>
-      <c r="G82" t="n">
-        <v>-639.7242830137967</v>
-      </c>
-      <c r="H82" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I82" t="n">
-        <v>0.000213381326830131</v>
-      </c>
-      <c r="J82" t="n">
-        <v>3.335520198697152e-08</v>
-      </c>
-      <c r="K82" t="n">
-        <v>0.9947867593616965</v>
-      </c>
-      <c r="L82" t="n">
-        <v>179</v>
-      </c>
-      <c r="M82" t="n">
-        <v>4.941018700000313</v>
-      </c>
-      <c r="N82" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="n">
-        <v>17</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E83" t="n">
-        <v>14</v>
-      </c>
-      <c r="F83" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="G83" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="H83" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I83" t="n">
-        <v>0.04093066525001632</v>
-      </c>
-      <c r="J83" t="n">
-        <v>6.398172825883034e-06</v>
-      </c>
-      <c r="K83" t="n">
-        <v>-3.777465056135922e-07</v>
-      </c>
-      <c r="L83" t="n">
-        <v>1451</v>
-      </c>
-      <c r="M83" t="n">
-        <v>2.635453100000177</v>
-      </c>
-      <c r="N83" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="n">
-        <v>18</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E84" t="n">
-        <v>14</v>
-      </c>
-      <c r="F84" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="G84" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="H84" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I84" t="n">
-        <v>0.04093066525001632</v>
-      </c>
-      <c r="J84" t="n">
-        <v>6.398172825883034e-06</v>
-      </c>
-      <c r="K84" t="n">
-        <v>-3.777465056135922e-07</v>
-      </c>
-      <c r="L84" t="n">
-        <v>1451</v>
-      </c>
-      <c r="M84" t="n">
-        <v>2.595588600000156</v>
-      </c>
-      <c r="N84" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="n">
-        <v>19</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E85" t="n">
-        <v>14</v>
-      </c>
-      <c r="F85" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="G85" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="H85" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I85" t="n">
-        <v>0.04093066525001632</v>
-      </c>
-      <c r="J85" t="n">
-        <v>6.398172825883034e-06</v>
-      </c>
-      <c r="K85" t="n">
-        <v>-3.777465056135922e-07</v>
-      </c>
-      <c r="L85" t="n">
-        <v>153</v>
-      </c>
-      <c r="M85" t="n">
-        <v>0.5478700999997272</v>
-      </c>
-      <c r="N85" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="n">
-        <v>20</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E86" t="n">
-        <v>14</v>
-      </c>
-      <c r="F86" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="G86" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="H86" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I86" t="n">
-        <v>0.04093066525001632</v>
-      </c>
-      <c r="J86" t="n">
-        <v>6.398172825883034e-06</v>
-      </c>
-      <c r="K86" t="n">
-        <v>-3.777465056135922e-07</v>
-      </c>
-      <c r="L86" t="n">
-        <v>179</v>
-      </c>
-      <c r="M86" t="n">
-        <v>3.155914200000097</v>
-      </c>
-      <c r="N86" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="n">
-        <v>21</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E87" t="n">
-        <v>14</v>
-      </c>
-      <c r="F87" t="n">
-        <v>-639.7242159339593</v>
-      </c>
-      <c r="G87" t="n">
-        <v>-639.7242159339593</v>
-      </c>
-      <c r="H87" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I87" t="n">
-        <v>0.06729321876264294</v>
-      </c>
-      <c r="J87" t="n">
-        <v>1.051909713715617e-05</v>
-      </c>
-      <c r="K87" t="n">
-        <v>-0.6440789264326543</v>
-      </c>
-      <c r="L87" t="n">
-        <v>1451</v>
-      </c>
-      <c r="M87" t="n">
-        <v>3.000794699999915</v>
-      </c>
-      <c r="N87" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="n">
-        <v>22</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E88" t="n">
-        <v>14</v>
-      </c>
-      <c r="F88" t="n">
-        <v>-639.7240257781056</v>
-      </c>
-      <c r="G88" t="n">
-        <v>-639.7242351048992</v>
-      </c>
-      <c r="H88" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I88" t="n">
-        <v>0.2574490724782663</v>
-      </c>
-      <c r="J88" t="n">
-        <v>4.024375488445252e-05</v>
-      </c>
-      <c r="K88" t="n">
-        <v>-5.289884812674799</v>
-      </c>
-      <c r="L88" t="n">
-        <v>1451</v>
-      </c>
-      <c r="M88" t="n">
-        <v>2.581269300000258</v>
-      </c>
-      <c r="N88" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="n">
-        <v>23</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E89" t="n">
-        <v>14</v>
-      </c>
-      <c r="F89" t="n">
-        <v>-639.7038001652395</v>
-      </c>
-      <c r="G89" t="n">
-        <v>-639.7038001652395</v>
-      </c>
-      <c r="H89" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I89" t="n">
-        <v>20.48306193853477</v>
-      </c>
-      <c r="J89" t="n">
-        <v>0.003201857812119484</v>
-      </c>
-      <c r="K89" t="n">
-        <v>-499.4333438223724</v>
-      </c>
-      <c r="L89" t="n">
-        <v>153</v>
-      </c>
-      <c r="M89" t="n">
-        <v>0.4916702000000441</v>
-      </c>
-      <c r="N89" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="n">
-        <v>24</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E90" t="n">
-        <v>14</v>
-      </c>
-      <c r="F90" t="n">
-        <v>-639.7240994374613</v>
-      </c>
-      <c r="G90" t="n">
-        <v>-639.7240994374613</v>
-      </c>
-      <c r="H90" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I90" t="n">
-        <v>0.1837897167433766</v>
-      </c>
-      <c r="J90" t="n">
-        <v>2.872952013267714e-05</v>
-      </c>
-      <c r="K90" t="n">
-        <v>-3.490271170689722</v>
-      </c>
-      <c r="L90" t="n">
-        <v>179</v>
-      </c>
-      <c r="M90" t="n">
-        <v>3.585163799999918</v>
-      </c>
-      <c r="N90" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="n">
-        <v>25</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E91" t="n">
-        <v>14</v>
-      </c>
-      <c r="F91" t="n">
-        <v>-639.7232132560886</v>
-      </c>
-      <c r="G91" t="n">
-        <v>-639.7232132560886</v>
-      </c>
-      <c r="H91" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I91" t="n">
-        <v>1.069971089464161</v>
-      </c>
-      <c r="J91" t="n">
-        <v>0.0001672550374462172</v>
-      </c>
-      <c r="K91" t="n">
-        <v>-25.14107264336669</v>
-      </c>
-      <c r="L91" t="n">
-        <v>1451</v>
-      </c>
-      <c r="M91" t="n">
-        <v>3.765098200000011</v>
-      </c>
-      <c r="N91" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="n">
-        <v>26</v>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E92" t="n">
-        <v>14</v>
-      </c>
-      <c r="F92" t="n">
-        <v>-639.7234348945376</v>
-      </c>
-      <c r="G92" t="n">
-        <v>-639.7242096712453</v>
-      </c>
-      <c r="H92" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I92" t="n">
-        <v>0.8483326404302716</v>
-      </c>
-      <c r="J92" t="n">
-        <v>0.0001326091040581951</v>
-      </c>
-      <c r="K92" t="n">
-        <v>-19.72609755309618</v>
-      </c>
-      <c r="L92" t="n">
-        <v>1451</v>
-      </c>
-      <c r="M92" t="n">
-        <v>3.872045100000378</v>
-      </c>
-      <c r="N92" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>27</v>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E93" t="n">
-        <v>14</v>
-      </c>
-      <c r="F93" t="n">
-        <v>-639.6307932658426</v>
-      </c>
-      <c r="G93" t="n">
-        <v>-639.6307932658426</v>
-      </c>
-      <c r="H93" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I93" t="n">
-        <v>93.48996133542187</v>
-      </c>
-      <c r="J93" t="n">
-        <v>0.01461410232292555</v>
-      </c>
-      <c r="K93" t="n">
-        <v>-2283.106453678781</v>
-      </c>
-      <c r="L93" t="n">
-        <v>153</v>
-      </c>
-      <c r="M93" t="n">
-        <v>0.8593877000002976</v>
-      </c>
-      <c r="N93" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>28</v>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E94" t="n">
-        <v>14</v>
-      </c>
-      <c r="F94" t="n">
-        <v>-639.7230688849096</v>
-      </c>
-      <c r="G94" t="n">
-        <v>-639.7230688849096</v>
-      </c>
-      <c r="H94" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I94" t="n">
-        <v>1.214342268440305</v>
-      </c>
-      <c r="J94" t="n">
-        <v>0.0001898227565029088</v>
-      </c>
-      <c r="K94" t="n">
-        <v>-28.66828708344459</v>
-      </c>
-      <c r="L94" t="n">
-        <v>179</v>
-      </c>
-      <c r="M94" t="n">
-        <v>3.608694699999887</v>
-      </c>
-      <c r="N94" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n">
-        <v>29</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E95" t="n">
-        <v>14</v>
-      </c>
-      <c r="F95" t="n">
-        <v>-639.7232818220903</v>
-      </c>
-      <c r="G95" t="n">
-        <v>-639.7232818220903</v>
-      </c>
-      <c r="H95" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I95" t="n">
-        <v>1.00140508777713</v>
-      </c>
-      <c r="J95" t="n">
-        <v>0.000156536982264516</v>
-      </c>
-      <c r="K95" t="n">
-        <v>-23.46589763292457</v>
-      </c>
-      <c r="L95" t="n">
-        <v>1451</v>
-      </c>
-      <c r="M95" t="n">
-        <v>3.458964200000082</v>
-      </c>
-      <c r="N95" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>30</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E96" t="n">
-        <v>14</v>
-      </c>
-      <c r="F96" t="n">
-        <v>-639.7241669187424</v>
-      </c>
-      <c r="G96" t="n">
-        <v>-639.7242102870636</v>
-      </c>
-      <c r="H96" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I96" t="n">
-        <v>0.1163084356221589</v>
-      </c>
-      <c r="J96" t="n">
-        <v>1.818102558737099e-05</v>
-      </c>
-      <c r="K96" t="n">
-        <v>-1.841597585742089</v>
-      </c>
-      <c r="L96" t="n">
-        <v>1451</v>
-      </c>
-      <c r="M96" t="n">
-        <v>3.891713099999834</v>
-      </c>
-      <c r="N96" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>31</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E97" t="n">
-        <v>14</v>
-      </c>
-      <c r="F97" t="n">
-        <v>-639.6987160058123</v>
-      </c>
-      <c r="G97" t="n">
-        <v>-639.6987160058123</v>
-      </c>
-      <c r="H97" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I97" t="n">
-        <v>25.56722136569078</v>
-      </c>
-      <c r="J97" t="n">
-        <v>0.003996600103518563</v>
-      </c>
-      <c r="K97" t="n">
-        <v>-623.6473363539851</v>
-      </c>
-      <c r="L97" t="n">
-        <v>153</v>
-      </c>
-      <c r="M97" t="n">
-        <v>1.045997799999896</v>
-      </c>
-      <c r="N97" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>32</v>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>PCU2</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E98" t="n">
-        <v>14</v>
-      </c>
-      <c r="F98" t="n">
-        <v>-639.7214750937679</v>
-      </c>
-      <c r="G98" t="n">
-        <v>-639.7214750937679</v>
-      </c>
-      <c r="H98" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I98" t="n">
-        <v>2.80813341009889</v>
-      </c>
-      <c r="J98" t="n">
-        <v>0.0004389599525490685</v>
-      </c>
-      <c r="K98" t="n">
-        <v>-67.60710554564839</v>
-      </c>
-      <c r="L98" t="n">
-        <v>179</v>
-      </c>
-      <c r="M98" t="n">
-        <v>3.345233099999859</v>
-      </c>
-      <c r="N98" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>33</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E99" t="n">
-        <v>3</v>
-      </c>
-      <c r="F99" t="n">
-        <v>-639.7242832271781</v>
-      </c>
-      <c r="G99" t="n">
-        <v>-639.7242832271787</v>
-      </c>
-      <c r="H99" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I99" t="n">
-        <v>1.13686837721616e-10</v>
-      </c>
-      <c r="J99" t="n">
-        <v>1.777122436999061e-14</v>
-      </c>
-      <c r="K99" t="n">
-        <v>1.000000002777548</v>
-      </c>
-      <c r="L99" t="n">
-        <v>351</v>
-      </c>
-      <c r="M99" t="n">
-        <v>6.646070499999951</v>
-      </c>
-      <c r="N99" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>34</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E100" t="n">
-        <v>3</v>
-      </c>
-      <c r="F100" t="n">
-        <v>-639.7242670873881</v>
-      </c>
-      <c r="G100" t="n">
-        <v>-639.7242823578147</v>
-      </c>
-      <c r="H100" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I100" t="n">
-        <v>0.01613978997738741</v>
-      </c>
-      <c r="J100" t="n">
-        <v>2.522929080629548e-06</v>
-      </c>
-      <c r="K100" t="n">
-        <v>0.6056796053631149</v>
-      </c>
-      <c r="L100" t="n">
-        <v>351</v>
-      </c>
-      <c r="M100" t="n">
-        <v>7.330478300000323</v>
-      </c>
-      <c r="N100" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>35</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E101" t="n">
-        <v>3</v>
-      </c>
-      <c r="F101" t="n">
-        <v>-639.7242585846084</v>
-      </c>
-      <c r="G101" t="n">
-        <v>-639.7242822948318</v>
-      </c>
-      <c r="H101" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I101" t="n">
-        <v>0.02464256965595268</v>
-      </c>
-      <c r="J101" t="n">
-        <v>3.852061005350589e-06</v>
-      </c>
-      <c r="K101" t="n">
-        <v>0.3979433558171294</v>
-      </c>
-      <c r="L101" t="n">
-        <v>153</v>
-      </c>
-      <c r="M101" t="n">
-        <v>2.779269299999669</v>
-      </c>
-      <c r="N101" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
-        <v>36</v>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E102" t="n">
-        <v>3</v>
-      </c>
-      <c r="F102" t="n">
-        <v>-639.7242801624316</v>
-      </c>
-      <c r="G102" t="n">
-        <v>-639.7242801624316</v>
-      </c>
-      <c r="H102" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I102" t="n">
-        <v>0.003064746465497592</v>
-      </c>
-      <c r="J102" t="n">
-        <v>4.790730234652111e-07</v>
-      </c>
-      <c r="K102" t="n">
-        <v>0.9251234348507532</v>
-      </c>
-      <c r="L102" t="n">
-        <v>179</v>
-      </c>
-      <c r="M102" t="n">
-        <v>13.19946549999986</v>
-      </c>
-      <c r="N102" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
-        <v>37</v>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E103" t="n">
-        <v>3</v>
-      </c>
-      <c r="F103" t="n">
-        <v>-639.7242832271784</v>
-      </c>
-      <c r="G103" t="n">
-        <v>-639.7242832271787</v>
-      </c>
-      <c r="H103" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I103" t="n">
-        <v>3.410605131648481e-10</v>
-      </c>
-      <c r="J103" t="n">
-        <v>5.331367310997184e-14</v>
-      </c>
-      <c r="K103" t="n">
-        <v>1.000000008332643</v>
-      </c>
-      <c r="L103" t="n">
-        <v>351</v>
-      </c>
-      <c r="M103" t="n">
-        <v>6.332708100000218</v>
-      </c>
-      <c r="N103" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
-        <v>38</v>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E104" t="n">
-        <v>3</v>
-      </c>
-      <c r="F104" t="n">
-        <v>-639.7238026042194</v>
-      </c>
-      <c r="G104" t="n">
-        <v>-639.7240758346587</v>
-      </c>
-      <c r="H104" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I104" t="n">
-        <v>0.4806229586620248</v>
-      </c>
-      <c r="J104" t="n">
-        <v>7.512970372758955e-05</v>
-      </c>
-      <c r="K104" t="n">
-        <v>-10.74237304182287</v>
-      </c>
-      <c r="L104" t="n">
-        <v>351</v>
-      </c>
-      <c r="M104" t="n">
-        <v>6.56686179999997</v>
-      </c>
-      <c r="N104" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>39</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E105" t="n">
-        <v>3</v>
-      </c>
-      <c r="F105" t="n">
-        <v>-639.7242183283884</v>
-      </c>
-      <c r="G105" t="n">
-        <v>-639.7242292714378</v>
-      </c>
-      <c r="H105" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I105" t="n">
-        <v>0.06489878967386176</v>
-      </c>
-      <c r="J105" t="n">
-        <v>1.014480634476947e-05</v>
-      </c>
-      <c r="K105" t="n">
-        <v>-0.5855792666142141</v>
-      </c>
-      <c r="L105" t="n">
-        <v>153</v>
-      </c>
-      <c r="M105" t="n">
-        <v>2.683258299999579</v>
-      </c>
-      <c r="N105" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>40</v>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E106" t="n">
-        <v>3</v>
-      </c>
-      <c r="F106" t="n">
-        <v>-639.7242270993788</v>
-      </c>
-      <c r="G106" t="n">
-        <v>-639.7242270993788</v>
-      </c>
-      <c r="H106" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I106" t="n">
-        <v>0.05612779921193578</v>
-      </c>
-      <c r="J106" t="n">
-        <v>8.773748423116174e-06</v>
-      </c>
-      <c r="K106" t="n">
-        <v>-0.3712902067721321</v>
-      </c>
-      <c r="L106" t="n">
-        <v>179</v>
-      </c>
-      <c r="M106" t="n">
-        <v>10.69913639999959</v>
-      </c>
-      <c r="N106" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>41</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E107" t="n">
-        <v>3</v>
-      </c>
-      <c r="F107" t="n">
-        <v>-639.7242832271778</v>
-      </c>
-      <c r="G107" t="n">
-        <v>-639.7242832271784</v>
-      </c>
-      <c r="H107" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I107" t="n">
-        <v>2.273736754432321e-10</v>
-      </c>
-      <c r="J107" t="n">
-        <v>3.554244873998122e-14</v>
-      </c>
-      <c r="K107" t="n">
-        <v>0.9999999944449043</v>
-      </c>
-      <c r="L107" t="n">
-        <v>351</v>
-      </c>
-      <c r="M107" t="n">
-        <v>6.964090400000259</v>
-      </c>
-      <c r="N107" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>42</v>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E108" t="n">
-        <v>3</v>
-      </c>
-      <c r="F108" t="n">
-        <v>-639.7228147828996</v>
-      </c>
-      <c r="G108" t="n">
-        <v>-639.7241894322134</v>
-      </c>
-      <c r="H108" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I108" t="n">
-        <v>1.46844427843007</v>
-      </c>
-      <c r="J108" t="n">
-        <v>0.0002295433074733851</v>
-      </c>
-      <c r="K108" t="n">
-        <v>-34.87639790753656</v>
-      </c>
-      <c r="L108" t="n">
-        <v>351</v>
-      </c>
-      <c r="M108" t="n">
-        <v>5.998219500000232</v>
-      </c>
-      <c r="N108" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>43</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E109" t="n">
-        <v>3</v>
-      </c>
-      <c r="F109" t="n">
-        <v>-639.7241914706718</v>
-      </c>
-      <c r="G109" t="n">
-        <v>-639.7242015511624</v>
-      </c>
-      <c r="H109" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I109" t="n">
-        <v>0.09175650620818487</v>
-      </c>
-      <c r="J109" t="n">
-        <v>1.43431332237861e-05</v>
-      </c>
-      <c r="K109" t="n">
-        <v>-1.241755424897422</v>
-      </c>
-      <c r="L109" t="n">
-        <v>153</v>
-      </c>
-      <c r="M109" t="n">
-        <v>4.236047299999882</v>
-      </c>
-      <c r="N109" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>44</v>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E110" t="n">
-        <v>3</v>
-      </c>
-      <c r="F110" t="n">
-        <v>-639.7241628866426</v>
-      </c>
-      <c r="G110" t="n">
-        <v>-639.7241628866426</v>
-      </c>
-      <c r="H110" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I110" t="n">
-        <v>0.1203405354317511</v>
-      </c>
-      <c r="J110" t="n">
-        <v>1.881131271501474e-05</v>
-      </c>
-      <c r="K110" t="n">
-        <v>-1.940108110994356</v>
-      </c>
-      <c r="L110" t="n">
-        <v>179</v>
-      </c>
-      <c r="M110" t="n">
-        <v>11.27448050000021</v>
-      </c>
-      <c r="N110" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>45</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E111" t="n">
-        <v>3</v>
-      </c>
-      <c r="F111" t="n">
-        <v>-639.7242832271779</v>
-      </c>
-      <c r="G111" t="n">
-        <v>-639.7242832271787</v>
-      </c>
-      <c r="H111" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I111" t="n">
-        <v>1.13686837721616e-10</v>
-      </c>
-      <c r="J111" t="n">
-        <v>1.777122436999061e-14</v>
-      </c>
-      <c r="K111" t="n">
-        <v>0.9999999972224521</v>
-      </c>
-      <c r="L111" t="n">
-        <v>351</v>
-      </c>
-      <c r="M111" t="n">
-        <v>6.095205699999951</v>
-      </c>
-      <c r="N111" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>46</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E112" t="n">
-        <v>3</v>
-      </c>
-      <c r="F112" t="n">
-        <v>-639.7165985912698</v>
-      </c>
-      <c r="G112" t="n">
-        <v>-639.7173498337671</v>
-      </c>
-      <c r="H112" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I112" t="n">
-        <v>7.684635908276505</v>
-      </c>
-      <c r="J112" t="n">
-        <v>0.001201241864621785</v>
-      </c>
-      <c r="K112" t="n">
-        <v>-186.7477134608215</v>
-      </c>
-      <c r="L112" t="n">
-        <v>351</v>
-      </c>
-      <c r="M112" t="n">
-        <v>5.603342700000212</v>
-      </c>
-      <c r="N112" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>47</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E113" t="n">
-        <v>3</v>
-      </c>
-      <c r="F113" t="n">
-        <v>-639.720200962994</v>
-      </c>
-      <c r="G113" t="n">
-        <v>-639.720200962994</v>
-      </c>
-      <c r="H113" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I113" t="n">
-        <v>4.082264184035012</v>
-      </c>
-      <c r="J113" t="n">
-        <v>0.0006381286893537107</v>
-      </c>
-      <c r="K113" t="n">
-        <v>-98.73611963451815</v>
-      </c>
-      <c r="L113" t="n">
-        <v>153</v>
-      </c>
-      <c r="M113" t="n">
-        <v>3.392699500000163</v>
-      </c>
-      <c r="N113" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>48</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>UCCSD</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E114" t="n">
-        <v>3</v>
-      </c>
-      <c r="F114" t="n">
-        <v>-639.7242643435908</v>
-      </c>
-      <c r="G114" t="n">
-        <v>-639.7242643435908</v>
-      </c>
-      <c r="H114" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I114" t="n">
-        <v>0.01888358724499994</v>
-      </c>
-      <c r="J114" t="n">
-        <v>2.951832178347063e-06</v>
-      </c>
-      <c r="K114" t="n">
-        <v>0.5386443327304212</v>
-      </c>
-      <c r="L114" t="n">
-        <v>179</v>
-      </c>
-      <c r="M114" t="n">
-        <v>12.2357963999998</v>
-      </c>
-      <c r="N114" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>49</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E115" t="n">
-        <v>9</v>
-      </c>
-      <c r="F115" t="n">
-        <v>-639.7242832067717</v>
-      </c>
-      <c r="G115" t="n">
-        <v>-639.7242832067717</v>
-      </c>
-      <c r="H115" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I115" t="n">
-        <v>2.040633262367919e-05</v>
-      </c>
-      <c r="J115" t="n">
-        <v>3.189863689515835e-09</v>
-      </c>
-      <c r="K115" t="n">
-        <v>0.9995014412737381</v>
-      </c>
-      <c r="L115" t="n">
-        <v>951</v>
-      </c>
-      <c r="M115" t="n">
-        <v>38.07708380000031</v>
-      </c>
-      <c r="N115" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>50</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E116" t="n">
-        <v>9</v>
-      </c>
-      <c r="F116" t="n">
-        <v>-639.7241400806973</v>
-      </c>
-      <c r="G116" t="n">
-        <v>-639.7242830296441</v>
-      </c>
-      <c r="H116" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I116" t="n">
-        <v>0.1431464806955773</v>
-      </c>
-      <c r="J116" t="n">
-        <v>2.237627747589243e-05</v>
-      </c>
-      <c r="K116" t="n">
-        <v>-2.497293139368243</v>
-      </c>
-      <c r="L116" t="n">
-        <v>951</v>
-      </c>
-      <c r="M116" t="n">
-        <v>36.49008110000022</v>
-      </c>
-      <c r="N116" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
-        <v>51</v>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E117" t="n">
-        <v>9</v>
-      </c>
-      <c r="F117" t="n">
-        <v>-639.7237304298095</v>
-      </c>
-      <c r="G117" t="n">
-        <v>-639.7242422965128</v>
-      </c>
-      <c r="H117" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I117" t="n">
-        <v>0.5527973685275356</v>
-      </c>
-      <c r="J117" t="n">
-        <v>8.641181568704449e-05</v>
-      </c>
-      <c r="K117" t="n">
-        <v>-12.50570712614033</v>
-      </c>
-      <c r="L117" t="n">
-        <v>153</v>
-      </c>
-      <c r="M117" t="n">
-        <v>5.613789199999701</v>
-      </c>
-      <c r="N117" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
-        <v>52</v>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E118" t="n">
-        <v>9</v>
-      </c>
-      <c r="F118" t="n">
-        <v>-639.7242780327507</v>
-      </c>
-      <c r="G118" t="n">
-        <v>-639.7242780327507</v>
-      </c>
-      <c r="H118" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I118" t="n">
-        <v>0.005194427330934559</v>
-      </c>
-      <c r="J118" t="n">
-        <v>8.119790771003015e-07</v>
-      </c>
-      <c r="K118" t="n">
-        <v>0.873091989553987</v>
-      </c>
-      <c r="L118" t="n">
-        <v>179</v>
-      </c>
-      <c r="M118" t="n">
-        <v>24.11561920000031</v>
-      </c>
-      <c r="N118" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
-        <v>53</v>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E119" t="n">
-        <v>9</v>
-      </c>
-      <c r="F119" t="n">
-        <v>-639.7234766132498</v>
-      </c>
-      <c r="G119" t="n">
-        <v>-639.7234766132498</v>
-      </c>
-      <c r="H119" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I119" t="n">
-        <v>0.8066139282618678</v>
-      </c>
-      <c r="J119" t="n">
-        <v>0.000126087745832125</v>
-      </c>
-      <c r="K119" t="n">
-        <v>-18.70684395258245</v>
-      </c>
-      <c r="L119" t="n">
-        <v>951</v>
-      </c>
-      <c r="M119" t="n">
-        <v>39.54827169999999</v>
-      </c>
-      <c r="N119" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>54</v>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E120" t="n">
-        <v>9</v>
-      </c>
-      <c r="F120" t="n">
-        <v>-639.7230609353746</v>
-      </c>
-      <c r="G120" t="n">
-        <v>-639.7242761906532</v>
-      </c>
-      <c r="H120" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I120" t="n">
-        <v>1.222291803401276</v>
-      </c>
-      <c r="J120" t="n">
-        <v>0.0001910654066835255</v>
-      </c>
-      <c r="K120" t="n">
-        <v>-28.86250669642479</v>
-      </c>
-      <c r="L120" t="n">
-        <v>951</v>
-      </c>
-      <c r="M120" t="n">
-        <v>39.87168580000025</v>
-      </c>
-      <c r="N120" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>55</v>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E121" t="n">
-        <v>9</v>
-      </c>
-      <c r="F121" t="n">
-        <v>-639.7239142307398</v>
-      </c>
-      <c r="G121" t="n">
-        <v>-639.7241372479696</v>
-      </c>
-      <c r="H121" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I121" t="n">
-        <v>0.3689964382829203</v>
-      </c>
-      <c r="J121" t="n">
-        <v>5.768054268965162e-05</v>
-      </c>
-      <c r="K121" t="n">
-        <v>-8.015161992019866</v>
-      </c>
-      <c r="L121" t="n">
-        <v>153</v>
-      </c>
-      <c r="M121" t="n">
-        <v>6.852394600000025</v>
-      </c>
-      <c r="N121" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="n">
-        <v>56</v>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E122" t="n">
-        <v>9</v>
-      </c>
-      <c r="F122" t="n">
-        <v>-639.7158237843419</v>
-      </c>
-      <c r="G122" t="n">
-        <v>-639.7158237843419</v>
-      </c>
-      <c r="H122" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I122" t="n">
-        <v>8.459442836169728</v>
-      </c>
-      <c r="J122" t="n">
-        <v>0.001322357624677758</v>
-      </c>
-      <c r="K122" t="n">
-        <v>-205.6774624849599</v>
-      </c>
-      <c r="L122" t="n">
-        <v>179</v>
-      </c>
-      <c r="M122" t="n">
-        <v>27.46157510000012</v>
-      </c>
-      <c r="N122" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="n">
-        <v>57</v>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E123" t="n">
-        <v>9</v>
-      </c>
-      <c r="F123" t="n">
-        <v>-639.7162946715627</v>
-      </c>
-      <c r="G123" t="n">
-        <v>-639.7162946715627</v>
-      </c>
-      <c r="H123" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I123" t="n">
-        <v>7.98855561538403</v>
-      </c>
-      <c r="J123" t="n">
-        <v>0.001248749785623996</v>
-      </c>
-      <c r="K123" t="n">
-        <v>-194.1729487961306</v>
-      </c>
-      <c r="L123" t="n">
-        <v>951</v>
-      </c>
-      <c r="M123" t="n">
-        <v>40.73785719999978</v>
-      </c>
-      <c r="N123" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>58</v>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E124" t="n">
-        <v>9</v>
-      </c>
-      <c r="F124" t="n">
-        <v>-639.7242620550909</v>
-      </c>
-      <c r="G124" t="n">
-        <v>-639.7242822148108</v>
-      </c>
-      <c r="H124" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I124" t="n">
-        <v>0.02117208714480512</v>
-      </c>
-      <c r="J124" t="n">
-        <v>3.309564401401114e-06</v>
-      </c>
-      <c r="K124" t="n">
-        <v>0.4827326892157314</v>
-      </c>
-      <c r="L124" t="n">
-        <v>951</v>
-      </c>
-      <c r="M124" t="n">
-        <v>40.91403280000031</v>
-      </c>
-      <c r="N124" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
-        <v>59</v>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E125" t="n">
-        <v>9</v>
-      </c>
-      <c r="F125" t="n">
-        <v>-639.7237433422893</v>
-      </c>
-      <c r="G125" t="n">
-        <v>-639.7242162018379</v>
-      </c>
-      <c r="H125" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I125" t="n">
-        <v>0.5398848887807617</v>
-      </c>
-      <c r="J125" t="n">
-        <v>8.439337116565865e-05</v>
-      </c>
-      <c r="K125" t="n">
-        <v>-12.19023498451877</v>
-      </c>
-      <c r="L125" t="n">
-        <v>153</v>
-      </c>
-      <c r="M125" t="n">
-        <v>6.533685299999888</v>
-      </c>
-      <c r="N125" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
-        <v>60</v>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E126" t="n">
-        <v>9</v>
-      </c>
-      <c r="F126" t="n">
-        <v>-639.7239016439627</v>
-      </c>
-      <c r="G126" t="n">
-        <v>-639.7239016439627</v>
-      </c>
-      <c r="H126" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I126" t="n">
-        <v>0.3815832153577503</v>
-      </c>
-      <c r="J126" t="n">
-        <v>5.964807423485643e-05</v>
-      </c>
-      <c r="K126" t="n">
-        <v>-8.322676706294784</v>
-      </c>
-      <c r="L126" t="n">
-        <v>179</v>
-      </c>
-      <c r="M126" t="n">
-        <v>26.65201989999969</v>
-      </c>
-      <c r="N126" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
-        <v>61</v>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="E127" t="n">
-        <v>9</v>
-      </c>
-      <c r="F127" t="n">
-        <v>-639.6871139122451</v>
-      </c>
-      <c r="G127" t="n">
-        <v>-639.6880108599083</v>
-      </c>
-      <c r="H127" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I127" t="n">
-        <v>37.16931493295306</v>
-      </c>
-      <c r="J127" t="n">
-        <v>0.005810208539442537</v>
-      </c>
-      <c r="K127" t="n">
-        <v>-907.1046874388896</v>
-      </c>
-      <c r="L127" t="n">
-        <v>951</v>
-      </c>
-      <c r="M127" t="n">
-        <v>39.4039557000001</v>
-      </c>
-      <c r="N127" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>62</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>ADAM</t>
-        </is>
-      </c>
-      <c r="E128" t="n">
-        <v>9</v>
-      </c>
-      <c r="F128" t="n">
-        <v>-639.7233128597095</v>
-      </c>
-      <c r="G128" t="n">
-        <v>-639.723922272774</v>
-      </c>
-      <c r="H128" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I128" t="n">
-        <v>0.9703674685397345</v>
-      </c>
-      <c r="J128" t="n">
-        <v>0.0001516852641023069</v>
-      </c>
-      <c r="K128" t="n">
-        <v>-22.70759989277888</v>
-      </c>
-      <c r="L128" t="n">
-        <v>951</v>
-      </c>
-      <c r="M128" t="n">
-        <v>37.31758059999993</v>
-      </c>
-      <c r="N128" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="n">
-        <v>63</v>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E129" t="n">
-        <v>9</v>
-      </c>
-      <c r="F129" t="n">
-        <v>-639.7232748551381</v>
-      </c>
-      <c r="G129" t="n">
-        <v>-639.7232748551381</v>
-      </c>
-      <c r="H129" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I129" t="n">
-        <v>1.008372039905225</v>
-      </c>
-      <c r="J129" t="n">
-        <v>0.0001576260377077376</v>
-      </c>
-      <c r="K129" t="n">
-        <v>-23.63611120549373</v>
-      </c>
-      <c r="L129" t="n">
-        <v>153</v>
-      </c>
-      <c r="M129" t="n">
-        <v>6.263222800000221</v>
-      </c>
-      <c r="N129" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="n">
-        <v>64</v>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>QNSPSA</t>
-        </is>
-      </c>
-      <c r="E130" t="n">
-        <v>9</v>
-      </c>
-      <c r="F130" t="n">
-        <v>-639.7215170097249</v>
-      </c>
-      <c r="G130" t="n">
-        <v>-639.7215170097249</v>
-      </c>
-      <c r="H130" t="n">
-        <v>-639.724283227178</v>
-      </c>
-      <c r="I130" t="n">
-        <v>2.766217453086028</v>
-      </c>
-      <c r="J130" t="n">
-        <v>0.0004324077615330561</v>
-      </c>
-      <c r="K130" t="n">
-        <v>-66.58303294408103</v>
-      </c>
-      <c r="L130" t="n">
-        <v>179</v>
-      </c>
-      <c r="M130" t="n">
-        <v>25.39412559999982</v>
-      </c>
-      <c r="N130" t="n">
-        <v>50</v>
-      </c>
-    </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I65">
     <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9814,7 +6127,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13128,13 +9441,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13146,7 +9459,7 @@
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
@@ -13248,28 +9561,28 @@
         <v>99</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>-639.2262965046541</v>
+        <v>-639.2262965047461</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>-639.7242422961749</v>
+        <v>-639.724242296175</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>499.3294707230689</v>
+        <v>499.3294706310962</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>0.07805369215306188</v>
+        <v>0.07805369213868499</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>-359.8709238536699</v>
+        <v>-359.8709237872002</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M2" s="9" t="n">
-        <v>31.31265560002066</v>
+        <v>49.57250350000004</v>
       </c>
       <c r="N2" t="n">
         <v>15</v>
@@ -13298,28 +9611,28 @@
         <v>99</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>-638.2758535574419</v>
+        <v>-638.275853557442</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>-638.2758535574419</v>
+        <v>-638.275853557442</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>1449.772417935264</v>
+        <v>1449.772417935151</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>0.2266240961857398</v>
+        <v>0.226624096185722</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>-1046.766539956595</v>
+        <v>-1046.766539956513</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M3" s="9" t="n">
-        <v>31.44986270001391</v>
+        <v>47.22263809999959</v>
       </c>
       <c r="N3" t="n">
         <v>15</v>
@@ -13348,28 +9661,28 @@
         <v>99</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>-638.1296701140368</v>
+        <v>-638.1296701140369</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-638.1296701140368</v>
+        <v>-638.1296701140369</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>1595.955861340371</v>
+        <v>1595.955861340258</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>0.2494750556392123</v>
+        <v>0.2494750556391946</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>-1152.414929180088</v>
+        <v>-1152.414929180006</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M4" s="9" t="n">
-        <v>30.97138329999871</v>
+        <v>50.58865920000017</v>
       </c>
       <c r="N4" t="n">
         <v>15</v>
@@ -13398,28 +9711,28 @@
         <v>99</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>-638.1276133345948</v>
+        <v>-638.1276133345949</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-638.1281625005904</v>
+        <v>-638.1281625005905</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>1598.012640782372</v>
+        <v>1598.012640782258</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>0.2497965652612264</v>
+        <v>0.2497965652612086</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-1153.901386401055</v>
+        <v>-1153.901386400973</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M5" s="9" t="n">
-        <v>31.55422890000045</v>
+        <v>45.64800199999991</v>
       </c>
       <c r="N5" t="n">
         <v>15</v>
@@ -13448,28 +9761,28 @@
         <v>46</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>-639.7242422965106</v>
+        <v>-639.7242422965107</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-639.7242422965106</v>
+        <v>-639.7242422965107</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>1.383678866545779</v>
+        <v>1.383678866432092</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>0.0002162925495498341</v>
+        <v>0.0002162925495320629</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>-3.286509334143046e-10</v>
+        <v>-2.464882000607285e-10</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>3.883212000015192</v>
+        <v>4.634261000000151</v>
       </c>
       <c r="N6" t="n">
         <v>15</v>
@@ -13498,28 +9811,28 @@
         <v>46</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>-639.5002502169669</v>
+        <v>-639.5002502169671</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-639.5002502169669</v>
+        <v>-639.5002502169671</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>225.3757584102232</v>
+        <v>225.3757584101095</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>0.03523006571240556</v>
+        <v>0.03523006571238779</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>-161.8815499993304</v>
+        <v>-161.8815499992483</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>3.531285800010664</v>
+        <v>5.280666199999814</v>
       </c>
       <c r="N7" t="n">
         <v>15</v>
@@ -13548,28 +9861,28 @@
         <v>46</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>-638.980100953308</v>
+        <v>-638.9801009533081</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-638.980100953308</v>
+        <v>-638.9801009533081</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>745.5250220691596</v>
+        <v>745.5250220690459</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>0.1165382457412851</v>
+        <v>0.1165382457412674</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>-537.7991681735434</v>
+        <v>-537.7991681734613</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>3.781571600004099</v>
+        <v>5.328885599999921</v>
       </c>
       <c r="N8" t="n">
         <v>15</v>
@@ -13598,28 +9911,28 @@
         <v>46</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>-639.5103694577066</v>
+        <v>-639.5103694577067</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-639.5103694577066</v>
+        <v>-639.5103694577067</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>215.2565176705821</v>
+        <v>215.2565176704684</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>0.03364825621021272</v>
+        <v>0.03364825621019495</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>-154.5682629443445</v>
+        <v>-154.5682629442624</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>4.773610000003828</v>
+        <v>5.439959600000293</v>
       </c>
       <c r="N9" t="n">
         <v>15</v>
@@ -13648,28 +9961,28 @@
         <v>117</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>-639.236391106611</v>
+        <v>-639.2363911066111</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-639.7242422961663</v>
+        <v>-639.7242422961664</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>489.2348687661752</v>
+        <v>489.2348687660615</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0.07647573411183088</v>
+        <v>0.07647573411181312</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>-352.5754435191241</v>
+        <v>-352.5754435190419</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>33.74752380000427</v>
+        <v>48.90217940000002</v>
       </c>
       <c r="N10" t="n">
         <v>15</v>
@@ -13698,28 +10011,28 @@
         <v>117</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>-638.6994958359577</v>
+        <v>-638.6994958359578</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-638.6994958359577</v>
+        <v>-638.6994958359578</v>
       </c>
       <c r="H11" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>1026.130139419479</v>
+        <v>1026.130139419365</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0.1604015999601326</v>
+        <v>0.1604015999601149</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>-740.5955859168049</v>
+        <v>-740.5955859167228</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>33.80914779999875</v>
+        <v>46.82227049999983</v>
       </c>
       <c r="N11" t="n">
         <v>15</v>
@@ -13748,28 +10061,28 @@
         <v>117</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>-638.7640011378496</v>
+        <v>-638.764001137852</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-638.7640011378496</v>
+        <v>-638.764001137852</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>961.6248375275518</v>
+        <v>961.6248375251644</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.1503183237440866</v>
+        <v>0.1503183237437134</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>-693.9768917438153</v>
+        <v>-693.9768917420898</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M12" s="9" t="n">
-        <v>31.96816399999079</v>
+        <v>48.78603320000002</v>
       </c>
       <c r="N12" t="n">
         <v>15</v>
@@ -13798,235 +10111,35 @@
         <v>117</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>-638.557883906349</v>
+        <v>-638.5578839063492</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-638.557883906349</v>
+        <v>-638.5578839063492</v>
       </c>
       <c r="H13" s="4" t="n">
         <v>-639.7256259753772</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>1167.742069028122</v>
+        <v>1167.742069028009</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.1825379540248507</v>
+        <v>0.1825379540248329</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>-842.9400916247696</v>
+        <v>-842.9400916246874</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>48</v>
       </c>
       <c r="M13" s="9" t="n">
-        <v>32.21742140001152</v>
+        <v>47.51859490000015</v>
       </c>
       <c r="N13" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>zero</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>855</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>-638.8015961129581</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>-639.7242422937636</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>-639.7256259753772</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>924.0298624190473</v>
-      </c>
-      <c r="J14" s="6" t="n">
-        <v>0.1444415894720799</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>-666.8065879762131</v>
-      </c>
-      <c r="L14" s="8" t="n">
-        <v>48</v>
-      </c>
-      <c r="M14" s="9" t="n">
-        <v>281.0532992000226</v>
-      </c>
-      <c r="N14" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>half</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>855</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>-638.5465845198298</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>-638.5583035978012</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>-639.7256259753772</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>1179.041455547349</v>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>0.1843042403920724</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>-851.1062830700057</v>
-      </c>
-      <c r="L15" s="8" t="n">
-        <v>48</v>
-      </c>
-      <c r="M15" s="9" t="n">
-        <v>242.1702005999978</v>
-      </c>
-      <c r="N15" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>855</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>-638.613712000059</v>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>-638.613712000059</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>-639.7256259753772</v>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>1111.913975318203</v>
-      </c>
-      <c r="J16" s="6" t="n">
-        <v>0.1738110730866673</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>-802.5925116493398</v>
-      </c>
-      <c r="L16" s="8" t="n">
-        <v>48</v>
-      </c>
-      <c r="M16" s="9" t="n">
-        <v>197.7058291999856</v>
-      </c>
-      <c r="N16" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>k-UpCCGSD</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>random</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>SPSA</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>855</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>-638.553163552329</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>-638.5553595890582</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>-639.7256259753772</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>1172.46242304816</v>
-      </c>
-      <c r="J17" s="6" t="n">
-        <v>0.183275825673003</v>
-      </c>
-      <c r="K17" s="7" t="n">
-        <v>-846.351543613895</v>
-      </c>
-      <c r="L17" s="8" t="n">
-        <v>48</v>
-      </c>
-      <c r="M17" s="9" t="n">
-        <v>248.8460880000202</v>
-      </c>
-      <c r="N17" t="n">
-        <v>15</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I17">
+  <conditionalFormatting sqref="I2:I13">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -14042,7 +10155,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14299,7 +10412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24754,7 +20867,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25520,7 +21633,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25966,4 +22079,387 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>IBM Quantum Device Calibrated Noisy Simulation &amp; Hardware Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Parameter</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Evaluated on Physical IBM Quantum QPU (ibm_fez)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Target Backend</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ibm_fez</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Job ID</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>daqph1uekp0c73ar40l0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ansatz Selected</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PCU2 (theta sweep [-0.10, +0.10])</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Parameters Optimized</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Transpiled 2-Qubit Gate Count</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Circuit Depth</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Exact Active Ground Energy (Ha)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>-639.72428323</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Measured Energy (Ha)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>-639.69642295</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Energy Error (mHa)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>27.81934671</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Shots</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>QPU Runtime (seconds)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>50.00000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Direct Job Dashboard</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://quantum.ibm.com/jobs/daqph1uekp0c73ar40l0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Physical QPU 5-Point Parameterized Energy Landscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Theta (rad)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Measured Energy (Ha)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Error (mHa)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Std Dev / Error Bar (Ha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>-639.6934113794631</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>30.8309170488883</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.00163840</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>-639.6951972857621</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>29.04501074999644</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.00162206</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>-639.6939549952303</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>30.28730128164625</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0.00160798</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>-639.6964229498001</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>27.81934671190811</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0.00159931</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>-639.6927483500383</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>31.49394647368808</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0.00163480</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Parameter Binding Transpilation Analysis at theta = 0</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>fake_fez</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>unbound_depth</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>unbound_2q_gates</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>bound_zero_depth</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>bound_zero_2q_gates</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>gate_reduction_at_zero</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
bug fx in represented values
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Config" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Results (2e, 2o)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Results (4e, 4o)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Results (6e, 6o)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Active Space Scaling" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Convergence" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Summary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Robustness" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Hardware" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Verification" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results (2e, 2o)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results (4e, 4o)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results (6e, 6o)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Space Scaling" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Convergence" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robustness" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardware" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -197,14 +197,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -228,7 +228,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -256,8 +256,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -283,8 +283,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -310,14 +310,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="11"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -341,7 +341,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -365,7 +365,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -389,7 +389,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -413,7 +413,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -437,7 +437,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -465,8 +465,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -492,8 +492,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -519,14 +519,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -550,7 +550,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -578,8 +578,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -605,8 +605,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -632,14 +632,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -662,14 +662,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -694,14 +694,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -726,14 +726,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -758,14 +758,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -793,8 +793,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -820,8 +820,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -847,7 +847,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -862,9 +862,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -884,9 +884,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -906,9 +906,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -928,9 +928,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1379,11 +1379,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RHF Energy (Ha)</t>
+          <t>Reference Determinant (Ha)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-639.7242422965273</v>
+        <v>-639.724242296512</v>
       </c>
     </row>
     <row r="15">
@@ -21571,7 +21571,7 @@
         <v>24</v>
       </c>
       <c r="E33" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F33" t="n">
         <v>18</v>

</xml_diff>

<commit_message>
phase J: documentation update, results.xlsx sheets, make round3 target
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -22,6 +22,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round 2 - Circuit Costs" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round 2 - Reconciled HW Jobs" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round 2 - Hardware Jobs V2" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round 3 - Review Verification" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round 3 - Zero Init" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round 3 - Perturbed Init" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round 3 - Random Init" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round 3 - Hardware Jobs V3" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,11 +35,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.00000000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.000000%"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="#,##0.0000"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -79,7 +85,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -114,6 +120,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00333f48"/>
         <bgColor rgb="00333f48"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
       </patternFill>
     </fill>
   </fills>
@@ -157,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -188,6 +200,10 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5934,12 +5950,8 @@
           <t>SKIPPED (&gt;12q)</t>
         </is>
       </c>
-      <c r="H32" s="13" t="n">
-        <v/>
-      </c>
-      <c r="I32" s="13" t="n">
-        <v/>
-      </c>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="13" t="n">
@@ -5969,12 +5981,8 @@
           <t>SKIPPED (&gt;12q)</t>
         </is>
       </c>
-      <c r="H33" s="13" t="n">
-        <v/>
-      </c>
-      <c r="I33" s="13" t="n">
-        <v/>
-      </c>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="13" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="13" t="n">
@@ -6004,12 +6012,8 @@
           <t>SKIPPED (&gt;12q)</t>
         </is>
       </c>
-      <c r="H34" s="13" t="n">
-        <v/>
-      </c>
-      <c r="I34" s="13" t="n">
-        <v/>
-      </c>
+      <c r="H34" s="13" t="n"/>
+      <c r="I34" s="13" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="13" t="n">
@@ -6039,12 +6043,8 @@
           <t>SKIPPED (&gt;12q)</t>
         </is>
       </c>
-      <c r="H35" s="13" t="n">
-        <v/>
-      </c>
-      <c r="I35" s="13" t="n">
-        <v/>
-      </c>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="13" t="n">
@@ -6074,12 +6074,8 @@
           <t>SKIPPED (&gt;12q)</t>
         </is>
       </c>
-      <c r="H36" s="13" t="n">
-        <v/>
-      </c>
-      <c r="I36" s="13" t="n">
-        <v/>
-      </c>
+      <c r="H36" s="13" t="n"/>
+      <c r="I36" s="13" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7785,6 +7781,1844 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="96" customWidth="1" min="2" max="2"/>
+    <col width="99" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Finding #</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Review Finding</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>DexcG/PCU2 zero-init reaches CASCI error 0.015 mHa; summary CSV only aggregated random init</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>VERIFIED &amp; REPRODUCED (DexcG reaches 0.0149 mHa, PCU2 reaches 0.0148 mHa)</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>converged flag was hardcoded True; maxiter=25 ended in unconverged state from random</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>VERIFIED &amp; FIXED (Schema v3 defines converged by optimizer success or energy plateau &lt; 1e-8)</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Mean % correlation distorted by outliers (-391.7%)</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>VERIFIED &amp; REPLACED (All reports now use median % correlation recovered)</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>run_live_hardware_job.py hardcoded params_1up (|theta| &lt;= 3e-4 repeating)</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>VERIFIED &amp; ELIMINATED (Params loaded dynamically from converged Schema v3 cache records)</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Fidelity discrepancy (0.0398 device mean for 2-CZ vs 0.00186 for 489-CZ; ignores 1Q, RO, T1)</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>VERIFIED &amp; UNIFIED (Single error model: actual transpiled CZ edges * readout * exp(-t/T1))</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Rotosolve text claimed omega=4 with points 0, pi/4, pi/2 (singular model)</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>VERIFIED &amp; CORRECTED (FFT peak at omega=2, formula E=a+b*cos(2th)+c*sin(2th))</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>figures/circuit_*.png dated Sep 21 showed old 2e2o circuits; silent GenericBackendV2 fallback</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>VERIFIED &amp; RESOLVED (2e2o preserved as _2e2o_4q.png, 8q rendered; mock fallback requires --mock)</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Ansatz</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Optimizer</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Error (mHa)</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>% Corr Recovered</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Evaluations</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Converged</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>Wall Time (s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>3-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="n">
+        <v>0.001032552177093748</v>
+      </c>
+      <c r="D2" s="19" t="n">
+        <v>99.98731378026709</v>
+      </c>
+      <c r="E2" s="12" t="n">
+        <v>35643</v>
+      </c>
+      <c r="F2" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" s="19" t="n">
+        <v>305.6523283999995</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>2-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="n">
+        <v>0.006425503784157627</v>
+      </c>
+      <c r="D3" s="19" t="n">
+        <v>99.92105449515401</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>22849</v>
+      </c>
+      <c r="F3" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="19" t="n">
+        <v>95.89332920000015</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>UCCSD-SA</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>0.007750064582978666</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>99.90478057726762</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>405</v>
+      </c>
+      <c r="F4" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>4.244708600002923</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>UCCSD</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>0.007750064696665504</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>99.90478057587082</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>848</v>
+      </c>
+      <c r="F5" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>7.549082900004578</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>PCU2</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>ADAM</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>0.01480145249388443</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>99.81814528808393</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>11181</v>
+      </c>
+      <c r="F6" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>513.8453265999997</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>0.01490982594987145</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>99.81681378202897</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>407</v>
+      </c>
+      <c r="F7" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>19.39156649999495</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>ADAM</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>0.01490982788254769</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>99.81681375828357</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>11101</v>
+      </c>
+      <c r="F8" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>476.9181931999919</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>PCU2</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>0.01490982879204239</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>99.81681374710928</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="F9" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>32.1334402999928</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>0.01490997090058954</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>99.81681200112462</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>630</v>
+      </c>
+      <c r="F10" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>25.25273779999407</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>COBYLA</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>0.01492040041739529</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>99.81668386121572</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>263</v>
+      </c>
+      <c r="F11" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>20.38543799999752</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>PCU2</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>COBYLA</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>0.01492300214067654</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>99.8166518957287</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>734</v>
+      </c>
+      <c r="F12" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>56.14701739999873</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>1-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>1.483564063278209</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>81.77252432165268</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>1443</v>
+      </c>
+      <c r="F13" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>5.481441600000835</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>QNSPSA</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>3.161021348319082</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>61.16282325017611</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>929</v>
+      </c>
+      <c r="F14" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>433.9585738000023</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>ROTOSOLVE</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>4.187866300867427</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>48.54672404604033</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>216</v>
+      </c>
+      <c r="F15" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>25.81774379999842</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>HF_baseline</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>8.139163587429721</v>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>-2.793575445525436e-09</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>0.001492899988079444</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>SPSA</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>55.16734738421292</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>-577.8011867331867</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>903</v>
+      </c>
+      <c r="F17" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>55.01823120001063</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Ansatz</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Optimizer</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>N Runs</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Median Error (mHa)</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>IQR (mHa)</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Min Error (mHa)</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>Max Error (mHa)</t>
+        </is>
+      </c>
+      <c r="H1" s="18" t="inlineStr">
+        <is>
+          <t>Median % Corr</t>
+        </is>
+      </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
+          <t>Success Rate (%)</t>
+        </is>
+      </c>
+      <c r="J1" s="18" t="inlineStr">
+        <is>
+          <t>Median Evaluations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>3-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="19" t="n">
+        <v>0.004414508566696895</v>
+      </c>
+      <c r="E2" s="19" t="n">
+        <v>0.0004556509338726755</v>
+      </c>
+      <c r="F2" s="19" t="n">
+        <v>0.004307597009756137</v>
+      </c>
+      <c r="G2" s="19" t="n">
+        <v>0.006903195526319905</v>
+      </c>
+      <c r="H2" s="19" t="n">
+        <v>99.94576213489998</v>
+      </c>
+      <c r="I2" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J2" s="12" t="n">
+        <v>35207</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>2-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D3" s="19" t="n">
+        <v>0.005898579047425301</v>
+      </c>
+      <c r="E3" s="19" t="n">
+        <v>0.003545556580775155</v>
+      </c>
+      <c r="F3" s="19" t="n">
+        <v>0.0009683039934316184</v>
+      </c>
+      <c r="G3" s="19" t="n">
+        <v>0.01284601239603944</v>
+      </c>
+      <c r="H3" s="19" t="n">
+        <v>99.9275284372377</v>
+      </c>
+      <c r="I3" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>23360</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>UCCSD-SA</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>0.007750064753508923</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>2.302158463862725e-09</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>0.005217119223743794</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>2.768240687373691</v>
+      </c>
+      <c r="H4" s="19" t="n">
+        <v>99.90478057517242</v>
+      </c>
+      <c r="I4" s="19" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>UCCSD</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>0.007750065549316787</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>3.467448550509289e-09</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>0.007750062309241912</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>2.328300568592567</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>99.90478056539492</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>PCU2</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>ADAM</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>0.0141875486860954</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>0.002334735427211854</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0.01118246723308403</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>0.0149402333136095</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>99.8256878789314</v>
+      </c>
+      <c r="I6" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>10921</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>PCU2</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>0.01490675799686869</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>2.638734031279455e-05</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>0.01448677198823134</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>0.01490982185714529</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>99.81685147574245</v>
+      </c>
+      <c r="I7" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>0.01490982691620957</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>1.790567694115452e-09</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>0.01490982231189264</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>0.01490983049734496</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>99.81681377015627</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>ADAM</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>0.01490982754148718</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>2.586375558166765e-09</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>0.01490982458562939</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>0.08452842871520261</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>99.81681376247394</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>11101</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>0.01491009385290454</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>1.246860392711824e-07</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>0.01490994429786952</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>0.01491032048761554</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>99.8168104904987</v>
+      </c>
+      <c r="I10" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>PCU2</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>COBYLA</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>0.0149104698721203</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>3.067441411985783e-05</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>0.01425489051598561</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>0.01500731980286218</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>99.8168058706233</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>COBYLA</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>0.01491968168920721</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>2.394472176092677e-06</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>0.01491585737767309</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>0.01492439696448855</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>99.8166926917077</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>1-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>1.483563134058841</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>2.699266588024329e-05</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>1.483451377453093</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>1.483802902953357</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>81.77253573829714</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>1554</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>ROTOSOLVE</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>7.442048135658297</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>6.97940003470876</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>2.297194659035995</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>594.5919121795669</v>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>8.564951964353723</v>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="12" t="n">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>QNSPSA</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>39.31550138150897</v>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>126.3235207583193</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>3.184432916896185</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>382.8777566629924</v>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>-383.0410515808637</v>
+      </c>
+      <c r="I15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>SPSA</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>49.13892384087148</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>6.411301197289276</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>35.88690340916401</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>57.64210015263416</v>
+      </c>
+      <c r="H16" s="19" t="n">
+        <v>-503.7343188203675</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>903</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Ansatz</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Optimizer</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>N Runs</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Median Error (mHa)</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>IQR (mHa)</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Min Error (mHa)</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>Max Error (mHa)</t>
+        </is>
+      </c>
+      <c r="H1" s="18" t="inlineStr">
+        <is>
+          <t>Median % Corr</t>
+        </is>
+      </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
+          <t>Success Rate (%)</t>
+        </is>
+      </c>
+      <c r="J1" s="18" t="inlineStr">
+        <is>
+          <t>Median Evaluations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" s="19" t="n">
+        <v>0.01490982720042666</v>
+      </c>
+      <c r="E2" s="19" t="n">
+        <v>1.904254531837068e-09</v>
+      </c>
+      <c r="F2" s="19" t="n">
+        <v>0.01490982481300307</v>
+      </c>
+      <c r="G2" s="19" t="n">
+        <v>0.01490982992891077</v>
+      </c>
+      <c r="H2" s="19" t="n">
+        <v>99.8168137666643</v>
+      </c>
+      <c r="I2" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J2" s="12" t="n">
+        <v>3589</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>2-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="19" t="n">
+        <v>0.01608508586059543</v>
+      </c>
+      <c r="E3" s="19" t="n">
+        <v>0.007677216473211956</v>
+      </c>
+      <c r="F3" s="19" t="n">
+        <v>0.006873881261526549</v>
+      </c>
+      <c r="G3" s="19" t="n">
+        <v>0.3651213644388918</v>
+      </c>
+      <c r="H3" s="19" t="n">
+        <v>99.8023742158729</v>
+      </c>
+      <c r="I3" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>23433</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>ADAM</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>0.0405739090751922</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>0.1654705139912949</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>0.01492957323989685</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>1.454236054314606</v>
+      </c>
+      <c r="H4" s="19" t="n">
+        <v>99.50149780575748</v>
+      </c>
+      <c r="I4" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>11101</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>1-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>1.483738377316968</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>1.398247803763297</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>0.0284137712469601</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>1.563401928478925</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>81.77038265148116</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>7548</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>UCCSD-SA</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>2.462747514130115</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>0.5956239216970971</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0.009409799076820491</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>3.044309699248515</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>69.7420074219613</v>
+      </c>
+      <c r="I6" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>14805</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>UCCSD</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>2.556818954076334</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>2.845123806736183</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>0.004798404802386358</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>3.029770171110613</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>68.5862198654348</v>
+      </c>
+      <c r="I7" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>17410</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>PCU2</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>L-BFGS-B</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>3.020277854432152</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0.7053587730183608</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>2.345552017004593</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>268.0973466417527</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>62.89203648417757</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>21027</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>PCU2</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>COBYLA</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>5.007113990416201</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>266.7119209272073</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>4.324726227309839</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>314.5328951424062</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>38.481221850742</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>COBYLA</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>532.3723442207893</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>20.94601106395544</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>0.01492157377924741</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>598.8955020562798</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>-6440.872885978941</v>
+      </c>
+      <c r="I10" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>594.0371353651699</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>28.63817730039386</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>534.3056167819213</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>646.7294936268217</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>-7198.503451868285</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>11101</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>QNSPSA</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>600.2829467105357</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>21.22347477117614</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>569.5122344114907</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>649.4941316393579</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>-7275.24120604227</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>ROTOSOLVE</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>607.2437936081769</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>27.58174360758403</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>585.79631551288</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>644.7753886739065</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>-7360.764083461593</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>DexcG</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>SPSA</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>613.1758577406003</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>39.68590881231648</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>578.3435052399</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>650.0693136925975</v>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>-7433.647053177925</v>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="12" t="n">
+        <v>903</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -11095,6 +12929,1596 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="103" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Experiment Name</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Resilience Type</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Calibration Time</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>QWC Circuits</t>
+        </is>
+      </c>
+      <c r="H1" s="18" t="inlineStr">
+        <is>
+          <t>2Q Gates</t>
+        </is>
+      </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
+          <t>Depth</t>
+        </is>
+      </c>
+      <c r="J1" s="18" t="inlineStr">
+        <is>
+          <t>Estimated Fidelity</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="inlineStr">
+        <is>
+          <t>Chemistry Signal</t>
+        </is>
+      </c>
+      <c r="L1" s="18" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>HF_baseline_2e2o</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="H2" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>RECOMMENDED: Reference baseline (2e2o)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>HF_baseline_2e2o</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="H3" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>RECOMMENDED: Reference baseline (2e2o)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>HF_baseline_2e2o</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>RECOMMENDED: Reference baseline (2e2o)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>HF_baseline_hard_4e4o</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>RECOMMENDED: Reference baseline (4e4o hard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>HF_baseline_hard_4e4o</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>RECOMMENDED: Reference baseline (4e4o hard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>HF_baseline_hard_4e4o</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>RECOMMENDED: Reference baseline (4e4o hard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>original_2e2o_parity_reduced</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="J8" s="19" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="K8" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>noise/mitigation test only: correlation signal is 0.04 mHa and cannot be resolved at this shot count</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>original_2e2o_parity_reduced</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="J9" s="19" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="K9" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>noise/mitigation test only: correlation signal is 0.04 mHa and cannot be resolved at this shot count</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>original_2e2o_parity_reduced</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="J10" s="19" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="K10" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>noise/mitigation test only: correlation signal is 0.04 mHa and cannot be resolved at this shot count</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_DexcG</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H11" s="12" t="n">
+        <v>1330</v>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>3724</v>
+      </c>
+      <c r="J11" s="19" t="n">
+        <v>0.0266</v>
+      </c>
+      <c r="K11" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0266 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_DexcG</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H12" s="12" t="n">
+        <v>1330</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>3724</v>
+      </c>
+      <c r="J12" s="19" t="n">
+        <v>0.0266</v>
+      </c>
+      <c r="K12" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0266 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_DexcG</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>1330</v>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>3724</v>
+      </c>
+      <c r="J13" s="19" t="n">
+        <v>0.0266</v>
+      </c>
+      <c r="K13" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0266 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_PCU2</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>1290</v>
+      </c>
+      <c r="I14" s="12" t="n">
+        <v>3577</v>
+      </c>
+      <c r="J14" s="19" t="n">
+        <v>0.0296</v>
+      </c>
+      <c r="K14" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0296 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_PCU2</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>1290</v>
+      </c>
+      <c r="I15" s="12" t="n">
+        <v>3577</v>
+      </c>
+      <c r="J15" s="19" t="n">
+        <v>0.0296</v>
+      </c>
+      <c r="K15" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0296 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_PCU2</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>1290</v>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>3577</v>
+      </c>
+      <c r="J16" s="19" t="n">
+        <v>0.0296</v>
+      </c>
+      <c r="K16" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0296 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_1-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>477</v>
+      </c>
+      <c r="I17" s="12" t="n">
+        <v>1253</v>
+      </c>
+      <c r="J17" s="19" t="n">
+        <v>0.2697</v>
+      </c>
+      <c r="K17" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.2697 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_1-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>477</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>1253</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>0.2697</v>
+      </c>
+      <c r="K18" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.2697 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_1-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>477</v>
+      </c>
+      <c r="I19" s="12" t="n">
+        <v>1253</v>
+      </c>
+      <c r="J19" s="19" t="n">
+        <v>0.2697</v>
+      </c>
+      <c r="K19" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.2697 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_2-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>971</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>2515</v>
+      </c>
+      <c r="J20" s="19" t="n">
+        <v>0.0756</v>
+      </c>
+      <c r="K20" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0756 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_2-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>971</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>2515</v>
+      </c>
+      <c r="J21" s="19" t="n">
+        <v>0.0756</v>
+      </c>
+      <c r="K21" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0756 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_2-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>971</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>2515</v>
+      </c>
+      <c r="J22" s="19" t="n">
+        <v>0.0756</v>
+      </c>
+      <c r="K22" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0756 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_3-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>1465</v>
+      </c>
+      <c r="I23" s="12" t="n">
+        <v>3731</v>
+      </c>
+      <c r="J23" s="19" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="K23" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0213 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_3-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H24" s="12" t="n">
+        <v>1465</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>3731</v>
+      </c>
+      <c r="J24" s="19" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="K24" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0213 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_3-UpCCGSD</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H25" s="12" t="n">
+        <v>1465</v>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>3731</v>
+      </c>
+      <c r="J25" s="19" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="K25" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0213 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_UCCSD</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H26" s="12" t="n">
+        <v>1409</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>3865</v>
+      </c>
+      <c r="J26" s="19" t="n">
+        <v>0.0217</v>
+      </c>
+      <c r="K26" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0217 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_UCCSD</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>1409</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>3865</v>
+      </c>
+      <c r="J27" s="19" t="n">
+        <v>0.0217</v>
+      </c>
+      <c r="K27" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0217 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_UCCSD</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>1409</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>3865</v>
+      </c>
+      <c r="J28" s="19" t="n">
+        <v>0.0217</v>
+      </c>
+      <c r="K28" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0217 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_UCCSD-SA</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>dynamical_decoupling</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>1413</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>3877</v>
+      </c>
+      <c r="J29" s="19" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="K29" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0214 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_UCCSD-SA</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>pauli_twirling</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H30" s="12" t="n">
+        <v>1413</v>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>3877</v>
+      </c>
+      <c r="J30" s="19" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="K30" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L30" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0214 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>hard_problem_UCCSD-SA</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>zne</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>ibm_marrakesh</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:15:23+05:30</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H31" s="12" t="n">
+        <v>1413</v>
+      </c>
+      <c r="I31" s="12" t="n">
+        <v>3877</v>
+      </c>
+      <c r="J31" s="19" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="K31" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L31" s="12" t="inlineStr">
+        <is>
+          <t>NOT RECOMMENDED: fidelity 0.0214 &lt; 0.3 threshold</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>